<commit_message>
added ASCII character to encoder
</commit_message>
<xml_diff>
--- a/Encoder data analysis/Encoder_analysis.xlsx
+++ b/Encoder data analysis/Encoder_analysis.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Desktop\T248 Decoding\C codes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dokumente\GitHub\Thrustmaster-T248-reverse-engineering\Encoder data analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CBA6649-78F1-4363-B7ED-092FC41D1BE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46AFB8D6-EB66-4A10-AF7E-2DA113825915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{EF999C88-1574-4865-9F82-FF9EA1A4DBD2}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1372" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1431" uniqueCount="130">
   <si>
     <t>timestamp</t>
   </si>
@@ -369,6 +369,93 @@
   </si>
   <si>
     <t>whole byte decides message</t>
+  </si>
+  <si>
+    <t>ASCII</t>
+  </si>
+  <si>
+    <t>" "</t>
+  </si>
+  <si>
+    <t>"E"</t>
+  </si>
+  <si>
+    <t>"1"</t>
+  </si>
+  <si>
+    <t>"2"</t>
+  </si>
+  <si>
+    <t>"3"</t>
+  </si>
+  <si>
+    <t>"4"</t>
+  </si>
+  <si>
+    <t>"+"</t>
+  </si>
+  <si>
+    <t>"-"</t>
+  </si>
+  <si>
+    <t>"P"</t>
+  </si>
+  <si>
+    <t>ASCII Length</t>
+  </si>
+  <si>
+    <t>ASCII Data</t>
+  </si>
+  <si>
+    <t>"     "</t>
+  </si>
+  <si>
+    <t>"E 1  "</t>
+  </si>
+  <si>
+    <t>"E 1 +"</t>
+  </si>
+  <si>
+    <t>"E 1 -"</t>
+  </si>
+  <si>
+    <t>"E 1 P"</t>
+  </si>
+  <si>
+    <t>"E 2  "</t>
+  </si>
+  <si>
+    <t>"E 2 +"</t>
+  </si>
+  <si>
+    <t>"E 2 -"</t>
+  </si>
+  <si>
+    <t>"E 2 P"</t>
+  </si>
+  <si>
+    <t>"E 3  "</t>
+  </si>
+  <si>
+    <t>"E 3 +"</t>
+  </si>
+  <si>
+    <t>"E 3 -"</t>
+  </si>
+  <si>
+    <t>"E 3 P"</t>
+  </si>
+  <si>
+    <t>"E 4  "</t>
+  </si>
+  <si>
+    <t>"E 4 +"</t>
+  </si>
+  <si>
+    <t>"E 4 -"</t>
+  </si>
+  <si>
+    <t>"E 4 P"</t>
   </si>
 </sst>
 </file>
@@ -710,7 +797,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -825,6 +912,58 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -870,12 +1009,21 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20 % - Akzent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -924,15 +1072,27 @@
   <dxfs count="18">
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor theme="4" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -1000,18 +1160,6 @@
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1062,20 +1210,20 @@
     <tableColumn id="3" xr3:uid="{654DF1FA-BDFD-4DD8-BB02-CAEAE5129DC0}" uniqueName="3" name="byte_1" queryTableFieldId="3" dataDxfId="16"/>
     <tableColumn id="4" xr3:uid="{4A07EA61-0E2B-4109-B662-32837551F715}" uniqueName="4" name="byte_2" queryTableFieldId="4" dataDxfId="15"/>
     <tableColumn id="5" xr3:uid="{BD664F6E-7B2D-4C8B-BB3D-1A0E22D0C8A1}" uniqueName="5" name="byte_3" queryTableFieldId="5" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{BCD67F6A-5BEE-493A-9AEA-6112EA05E14D}" uniqueName="6" name="byte_4" queryTableFieldId="6" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{47B18A3A-F003-4575-BD92-CBD286EADAF1}" uniqueName="7" name="byte_5" queryTableFieldId="7" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{5651D576-F2B9-4DA4-A57E-92606FBE8E3B}" uniqueName="8" name="byte_6" queryTableFieldId="8" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{5DAEAE6B-9C8E-49B8-9971-8F894474AAAA}" uniqueName="9" name="byte_7" queryTableFieldId="9" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{945A29B0-8B22-48F6-A986-B55E6E0CB240}" uniqueName="10" name="byte_8" queryTableFieldId="10" dataDxfId="5"/>
-    <tableColumn id="11" xr3:uid="{6B9E6EA5-3354-4B5A-9516-B6843C3BAF1E}" uniqueName="11" name="byte_9" queryTableFieldId="11" dataDxfId="4"/>
-    <tableColumn id="12" xr3:uid="{A97E2A78-B181-428B-A84C-E9BA8B8183EA}" uniqueName="12" name="byte_10" queryTableFieldId="12" dataDxfId="3"/>
-    <tableColumn id="13" xr3:uid="{5645FC6A-A5CF-4C65-BD82-6D3599CB51EF}" uniqueName="13" name="byte_11" queryTableFieldId="13" dataDxfId="2"/>
-    <tableColumn id="14" xr3:uid="{1291BB16-8527-4CBC-94D2-10703A5B7099}" uniqueName="14" name="byte_12" queryTableFieldId="14" dataDxfId="0"/>
-    <tableColumn id="15" xr3:uid="{14194924-ECFE-4865-9EB4-B3BAB41410D8}" uniqueName="15" name="byte_13" queryTableFieldId="15" dataDxfId="1"/>
-    <tableColumn id="16" xr3:uid="{4D2A8C4C-D766-47B8-BC45-D6D21AEAE4D0}" uniqueName="16" name="byte_14" queryTableFieldId="16" dataDxfId="13"/>
-    <tableColumn id="17" xr3:uid="{75741803-4CE8-4306-BB06-682A6DD255D0}" uniqueName="17" name="byte_15" queryTableFieldId="17" dataDxfId="12"/>
-    <tableColumn id="18" xr3:uid="{16E2CBC7-555A-4EB3-810A-EE0C55392CA7}" uniqueName="18" name="byte_16" queryTableFieldId="18" dataDxfId="11"/>
-    <tableColumn id="19" xr3:uid="{F74D354D-42D3-46EE-87EE-4B19132D80AB}" uniqueName="19" name="byte_17" queryTableFieldId="19" dataDxfId="10"/>
+    <tableColumn id="6" xr3:uid="{BCD67F6A-5BEE-493A-9AEA-6112EA05E14D}" uniqueName="6" name="byte_4" queryTableFieldId="6" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{47B18A3A-F003-4575-BD92-CBD286EADAF1}" uniqueName="7" name="byte_5" queryTableFieldId="7" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{5651D576-F2B9-4DA4-A57E-92606FBE8E3B}" uniqueName="8" name="byte_6" queryTableFieldId="8" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{5DAEAE6B-9C8E-49B8-9971-8F894474AAAA}" uniqueName="9" name="byte_7" queryTableFieldId="9" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{945A29B0-8B22-48F6-A986-B55E6E0CB240}" uniqueName="10" name="byte_8" queryTableFieldId="10" dataDxfId="9"/>
+    <tableColumn id="11" xr3:uid="{6B9E6EA5-3354-4B5A-9516-B6843C3BAF1E}" uniqueName="11" name="byte_9" queryTableFieldId="11" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{A97E2A78-B181-428B-A84C-E9BA8B8183EA}" uniqueName="12" name="byte_10" queryTableFieldId="12" dataDxfId="7"/>
+    <tableColumn id="13" xr3:uid="{5645FC6A-A5CF-4C65-BD82-6D3599CB51EF}" uniqueName="13" name="byte_11" queryTableFieldId="13" dataDxfId="6"/>
+    <tableColumn id="14" xr3:uid="{1291BB16-8527-4CBC-94D2-10703A5B7099}" uniqueName="14" name="byte_12" queryTableFieldId="14" dataDxfId="5"/>
+    <tableColumn id="15" xr3:uid="{14194924-ECFE-4865-9EB4-B3BAB41410D8}" uniqueName="15" name="byte_13" queryTableFieldId="15" dataDxfId="4"/>
+    <tableColumn id="16" xr3:uid="{4D2A8C4C-D766-47B8-BC45-D6D21AEAE4D0}" uniqueName="16" name="byte_14" queryTableFieldId="16" dataDxfId="3"/>
+    <tableColumn id="17" xr3:uid="{75741803-4CE8-4306-BB06-682A6DD255D0}" uniqueName="17" name="byte_15" queryTableFieldId="17" dataDxfId="2"/>
+    <tableColumn id="18" xr3:uid="{16E2CBC7-555A-4EB3-810A-EE0C55392CA7}" uniqueName="18" name="byte_16" queryTableFieldId="18" dataDxfId="1"/>
+    <tableColumn id="19" xr3:uid="{F74D354D-42D3-46EE-87EE-4B19132D80AB}" uniqueName="19" name="byte_17" queryTableFieldId="19" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1398,7 +1546,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E60B99F-BCDF-4887-BAA4-2EB8237F6FE8}">
-  <dimension ref="A1:U147"/>
+  <dimension ref="A1:W147"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
@@ -3344,7 +3492,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -3403,12 +3551,27 @@
         <v>33</v>
       </c>
     </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="H34" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="J34" s="5"/>
+      <c r="K34" s="5"/>
+      <c r="L34" s="5"/>
+      <c r="M34" s="6"/>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V36" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>36</v>
       </c>
@@ -3472,8 +3635,11 @@
       <c r="U37" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V37" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
         <v>36</v>
       </c>
@@ -3534,8 +3700,11 @@
       <c r="U38" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V38" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
         <v>36</v>
       </c>
@@ -3596,8 +3765,11 @@
       <c r="U39" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V39" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B40" t="s">
         <v>36</v>
       </c>
@@ -3658,8 +3830,11 @@
       <c r="U40" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V40" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B41" t="s">
         <v>36</v>
       </c>
@@ -3720,8 +3895,11 @@
       <c r="U41" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V41" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="42" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B42" t="s">
         <v>36</v>
       </c>
@@ -3782,8 +3960,11 @@
       <c r="U42" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V42" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="43" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B43" t="s">
         <v>36</v>
       </c>
@@ -3844,8 +4025,11 @@
       <c r="U43" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V43" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
         <v>36</v>
       </c>
@@ -3906,8 +4090,11 @@
       <c r="U44" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V44" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B45" t="s">
         <v>36</v>
       </c>
@@ -3968,8 +4155,11 @@
       <c r="U45" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V45" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="46" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B46" t="s">
         <v>36</v>
       </c>
@@ -4030,8 +4220,11 @@
       <c r="U46" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V46" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="47" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B47" t="s">
         <v>36</v>
       </c>
@@ -4092,8 +4285,11 @@
       <c r="U47" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V47" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="48" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B48" t="s">
         <v>36</v>
       </c>
@@ -4154,8 +4350,11 @@
       <c r="U48" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V48" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="50" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>32</v>
       </c>
@@ -4214,7 +4413,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>58</v>
       </c>
@@ -4278,8 +4477,11 @@
       <c r="U53" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V53" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="54" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B54" t="s">
         <v>35</v>
       </c>
@@ -4340,8 +4542,11 @@
       <c r="U54" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V54" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="55" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B55" t="s">
         <v>37</v>
       </c>
@@ -4402,8 +4607,11 @@
       <c r="U55" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V55" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="56" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B56" t="s">
         <v>38</v>
       </c>
@@ -4464,8 +4672,11 @@
       <c r="U56" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="58" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V56" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="58" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>32</v>
       </c>
@@ -4524,7 +4735,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="59" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:22" x14ac:dyDescent="0.25">
       <c r="I59" s="2"/>
       <c r="K59" s="2"/>
       <c r="M59" s="2"/>
@@ -4532,7 +4743,7 @@
       <c r="O59" s="2"/>
       <c r="P59" s="2"/>
     </row>
-    <row r="61" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>42</v>
       </c>
@@ -4596,8 +4807,11 @@
       <c r="U61" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="62" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V61" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="62" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
         <v>44</v>
       </c>
@@ -4658,8 +4872,11 @@
       <c r="U62" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="63" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V62" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="63" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
         <v>45</v>
       </c>
@@ -4720,8 +4937,11 @@
       <c r="U63" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="64" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V63" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="64" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
         <v>46</v>
       </c>
@@ -4782,8 +5002,11 @@
       <c r="U64" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="66" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V64" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="66" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>32</v>
       </c>
@@ -4842,7 +5065,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="69" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>60</v>
       </c>
@@ -4906,8 +5129,11 @@
       <c r="U69" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="70" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V69" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="70" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B70" t="s">
         <v>49</v>
       </c>
@@ -4968,8 +5194,11 @@
       <c r="U70" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="71" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V70" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="71" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B71" t="s">
         <v>50</v>
       </c>
@@ -5030,8 +5259,11 @@
       <c r="U71" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="72" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V71" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="72" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B72" t="s">
         <v>51</v>
       </c>
@@ -5092,8 +5324,11 @@
       <c r="U72" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="74" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V72" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="74" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>32</v>
       </c>
@@ -5152,7 +5387,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="77" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>61</v>
       </c>
@@ -5216,8 +5451,11 @@
       <c r="U77" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="78" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V77" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="78" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B78" t="s">
         <v>53</v>
       </c>
@@ -5278,8 +5516,11 @@
       <c r="U78" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="79" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V78" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="79" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B79" t="s">
         <v>54</v>
       </c>
@@ -5340,8 +5581,11 @@
       <c r="U79" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="80" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V79" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="80" spans="1:22" x14ac:dyDescent="0.25">
       <c r="B80" t="s">
         <v>55</v>
       </c>
@@ -5402,8 +5646,11 @@
       <c r="U80" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="82" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V80" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="82" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>32</v>
       </c>
@@ -5462,7 +5709,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="85" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>62</v>
       </c>
@@ -5526,8 +5773,11 @@
       <c r="U85" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="86" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V85" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="86" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B86" t="s">
         <v>43</v>
       </c>
@@ -5588,8 +5838,11 @@
       <c r="U86" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="87" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V86" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="87" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B87" t="s">
         <v>47</v>
       </c>
@@ -5650,8 +5903,11 @@
       <c r="U87" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="88" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V87" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="88" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B88" t="s">
         <v>52</v>
       </c>
@@ -5712,8 +5968,11 @@
       <c r="U88" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="90" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V88" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="90" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>32</v>
       </c>
@@ -5772,7 +6031,10 @@
         <v>33</v>
       </c>
     </row>
-    <row r="93" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="W92" s="1"/>
+    </row>
+    <row r="93" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>63</v>
       </c>
@@ -5836,8 +6098,11 @@
       <c r="U93" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="94" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V93" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="94" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B94" t="s">
         <v>44</v>
       </c>
@@ -5898,8 +6163,11 @@
       <c r="U94" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="95" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V94" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="95" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B95" t="s">
         <v>49</v>
       </c>
@@ -5960,8 +6228,11 @@
       <c r="U95" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="96" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V95" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="96" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B96" t="s">
         <v>53</v>
       </c>
@@ -6022,8 +6293,11 @@
       <c r="U96" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="98" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V96" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="98" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>32</v>
       </c>
@@ -6082,7 +6356,10 @@
         <v>33</v>
       </c>
     </row>
-    <row r="101" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="W100" s="1"/>
+    </row>
+    <row r="101" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>64</v>
       </c>
@@ -6146,8 +6423,11 @@
       <c r="U101" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="102" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V101" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="102" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B102" t="s">
         <v>45</v>
       </c>
@@ -6208,8 +6488,11 @@
       <c r="U102" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="103" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V102" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="103" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B103" t="s">
         <v>50</v>
       </c>
@@ -6270,8 +6553,11 @@
       <c r="U103" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="104" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V103" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="104" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B104" t="s">
         <v>54</v>
       </c>
@@ -6332,8 +6618,11 @@
       <c r="U104" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="106" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V104" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="106" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>32</v>
       </c>
@@ -6392,7 +6681,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="108" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>65</v>
       </c>
@@ -6456,8 +6745,12 @@
       <c r="U108" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="109" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V108" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="W108" s="1"/>
+    </row>
+    <row r="109" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B109" t="s">
         <v>46</v>
       </c>
@@ -6518,8 +6811,11 @@
       <c r="U109" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="110" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V109" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="110" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B110" t="s">
         <v>51</v>
       </c>
@@ -6580,8 +6876,11 @@
       <c r="U110" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="111" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V110" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="111" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B111" t="s">
         <v>55</v>
       </c>
@@ -6642,8 +6941,11 @@
       <c r="U111" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="113" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="V111" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="113" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>32</v>
       </c>
@@ -6702,7 +7004,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="116" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B116" t="s">
         <v>66</v>
       </c>
@@ -6722,15 +7024,18 @@
       <c r="L116" s="1"/>
       <c r="M116" s="1"/>
       <c r="N116" s="1"/>
-      <c r="O116" s="1"/>
+      <c r="O116" s="1" t="s">
+        <v>101</v>
+      </c>
       <c r="P116" s="1"/>
       <c r="Q116" s="1"/>
       <c r="R116" s="1"/>
       <c r="S116" s="1"/>
       <c r="T116" s="1"/>
       <c r="U116" s="1"/>
-    </row>
-    <row r="117" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="W116" s="1"/>
+    </row>
+    <row r="117" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>97</v>
       </c>
@@ -6746,42 +7051,35 @@
       <c r="E117" s="1"/>
       <c r="F117" s="1"/>
       <c r="G117" s="1"/>
-      <c r="H117" s="4" t="str">
+      <c r="H117" t="str">
         <f>HEX2BIN(C117,8)</f>
         <v>00100000</v>
       </c>
-      <c r="J117" s="4" t="str" cm="1">
+      <c r="J117" t="str" cm="1">
         <f t="array" ref="J117">_xlfn.TEXTJOIN("", TRUE, MID(H117, _xlfn.SEQUENCE(LEN(H117), 1, LEN(H117), -1), 1))</f>
         <v>00000100</v>
       </c>
-      <c r="K117" s="4"/>
-      <c r="L117" s="4" t="str">
+      <c r="L117" t="str">
         <f>MID($J117, COLUMN(K117), 1)</f>
         <v/>
       </c>
-      <c r="M117" s="4" t="str">
+      <c r="M117" t="str">
         <f>MID($J117, COLUMN(L117), 1)</f>
         <v/>
       </c>
-      <c r="N117" s="4" t="str">
+      <c r="N117" t="str">
         <f>MID($J117, COLUMN(M117), 1)</f>
         <v/>
       </c>
-      <c r="O117" s="4" t="str">
-        <f>MID($J117, COLUMN(N117), 1)</f>
-        <v/>
-      </c>
-      <c r="P117" s="4" t="str">
+      <c r="O117" t="s">
+        <v>102</v>
+      </c>
+      <c r="P117" t="str">
         <f>MID($J117, COLUMN(O117), 1)</f>
         <v/>
       </c>
-      <c r="Q117" s="4"/>
-      <c r="R117" s="4"/>
-      <c r="S117" s="4"/>
-      <c r="T117" s="4"/>
-      <c r="U117" s="4"/>
-    </row>
-    <row r="118" spans="1:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="118" spans="1:23" x14ac:dyDescent="0.25">
       <c r="C118" s="1" t="s">
         <v>41</v>
       </c>
@@ -6791,12 +7089,12 @@
       <c r="E118" s="1"/>
       <c r="F118" s="1"/>
       <c r="G118" s="1"/>
-      <c r="H118" s="4" t="str">
+      <c r="H118" t="str">
         <f t="shared" ref="H118:H140" si="0">HEX2BIN(C118,8)</f>
         <v>01000101</v>
       </c>
       <c r="I118" s="1"/>
-      <c r="J118" s="4" t="str" cm="1">
+      <c r="J118" t="str" cm="1">
         <f t="array" ref="J118">_xlfn.TEXTJOIN("", TRUE, MID(H118, _xlfn.SEQUENCE(LEN(H118), 1, LEN(H118), -1), 1))</f>
         <v>10100010</v>
       </c>
@@ -6804,7 +7102,9 @@
       <c r="L118" s="1"/>
       <c r="M118" s="1"/>
       <c r="N118" s="1"/>
-      <c r="O118" s="1"/>
+      <c r="O118" s="1" t="s">
+        <v>103</v>
+      </c>
       <c r="P118" s="1"/>
       <c r="Q118" s="1"/>
       <c r="R118" s="1"/>
@@ -6812,15 +7112,13 @@
       <c r="T118" s="1"/>
       <c r="U118" s="1"/>
     </row>
-    <row r="119" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:23" x14ac:dyDescent="0.25">
       <c r="C119" s="1"/>
       <c r="D119" s="1"/>
       <c r="E119" s="1"/>
       <c r="F119" s="1"/>
       <c r="G119" s="1"/>
-      <c r="H119" s="4"/>
       <c r="I119" s="1"/>
-      <c r="J119" s="4"/>
       <c r="K119" s="1"/>
       <c r="L119" s="1"/>
       <c r="M119" s="1"/>
@@ -6833,7 +7131,7 @@
       <c r="T119" s="1"/>
       <c r="U119" s="1"/>
     </row>
-    <row r="120" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>90</v>
       </c>
@@ -6849,12 +7147,12 @@
       <c r="E120" s="1"/>
       <c r="F120" s="1"/>
       <c r="G120" s="1"/>
-      <c r="H120" s="4" t="str">
+      <c r="H120" t="str">
         <f t="shared" si="0"/>
         <v>00100000</v>
       </c>
       <c r="I120" s="1"/>
-      <c r="J120" s="4" t="str" cm="1">
+      <c r="J120" t="str" cm="1">
         <f t="array" ref="J120">_xlfn.TEXTJOIN("", TRUE, MID(H120, _xlfn.SEQUENCE(LEN(H120), 1, LEN(H120), -1), 1))</f>
         <v>00000100</v>
       </c>
@@ -6862,7 +7160,9 @@
       <c r="L120" s="1"/>
       <c r="M120" s="1"/>
       <c r="N120" s="1"/>
-      <c r="O120" s="1"/>
+      <c r="O120" t="s">
+        <v>102</v>
+      </c>
       <c r="P120" s="1"/>
       <c r="Q120" s="1"/>
       <c r="R120" s="1"/>
@@ -6870,7 +7170,7 @@
       <c r="T120" s="1"/>
       <c r="U120" s="1"/>
     </row>
-    <row r="121" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:23" x14ac:dyDescent="0.25">
       <c r="C121" s="1" t="s">
         <v>70</v>
       </c>
@@ -6880,12 +7180,12 @@
       <c r="E121" s="1"/>
       <c r="F121" s="1"/>
       <c r="G121" s="1"/>
-      <c r="H121" s="4" t="str">
+      <c r="H121" t="str">
         <f t="shared" si="0"/>
         <v>00110001</v>
       </c>
       <c r="I121" s="1"/>
-      <c r="J121" s="4" t="str" cm="1">
+      <c r="J121" t="str" cm="1">
         <f t="array" ref="J121">_xlfn.TEXTJOIN("", TRUE, MID(H121, _xlfn.SEQUENCE(LEN(H121), 1, LEN(H121), -1), 1))</f>
         <v>10001100</v>
       </c>
@@ -6895,7 +7195,9 @@
       </c>
       <c r="M121" s="1"/>
       <c r="N121" s="1"/>
-      <c r="O121" s="1"/>
+      <c r="O121" s="1" t="s">
+        <v>104</v>
+      </c>
       <c r="P121" s="1"/>
       <c r="Q121" s="1"/>
       <c r="R121" s="1"/>
@@ -6903,7 +7205,7 @@
       <c r="T121" s="1"/>
       <c r="U121" s="1"/>
     </row>
-    <row r="122" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:23" x14ac:dyDescent="0.25">
       <c r="C122" s="1" t="s">
         <v>72</v>
       </c>
@@ -6913,12 +7215,12 @@
       <c r="E122" s="1"/>
       <c r="F122" s="1"/>
       <c r="G122" s="1"/>
-      <c r="H122" s="4" t="str">
+      <c r="H122" t="str">
         <f t="shared" si="0"/>
         <v>00110010</v>
       </c>
       <c r="I122" s="1"/>
-      <c r="J122" s="4" t="str" cm="1">
+      <c r="J122" t="str" cm="1">
         <f t="array" ref="J122">_xlfn.TEXTJOIN("", TRUE, MID(H122, _xlfn.SEQUENCE(LEN(H122), 1, LEN(H122), -1), 1))</f>
         <v>01001100</v>
       </c>
@@ -6926,7 +7228,9 @@
       <c r="L122" s="1"/>
       <c r="M122" s="1"/>
       <c r="N122" s="1"/>
-      <c r="O122" s="1"/>
+      <c r="O122" s="1" t="s">
+        <v>105</v>
+      </c>
       <c r="P122" s="1"/>
       <c r="Q122" s="1"/>
       <c r="R122" s="1"/>
@@ -6934,7 +7238,7 @@
       <c r="T122" s="1"/>
       <c r="U122" s="1"/>
     </row>
-    <row r="123" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:23" x14ac:dyDescent="0.25">
       <c r="C123" s="1" t="s">
         <v>74</v>
       </c>
@@ -6944,12 +7248,12 @@
       <c r="E123" s="1"/>
       <c r="F123" s="1"/>
       <c r="G123" s="1"/>
-      <c r="H123" s="4" t="str">
+      <c r="H123" t="str">
         <f t="shared" si="0"/>
         <v>00110011</v>
       </c>
       <c r="I123" s="1"/>
-      <c r="J123" s="4" t="str" cm="1">
+      <c r="J123" t="str" cm="1">
         <f t="array" ref="J123">_xlfn.TEXTJOIN("", TRUE, MID(H123, _xlfn.SEQUENCE(LEN(H123), 1, LEN(H123), -1), 1))</f>
         <v>11001100</v>
       </c>
@@ -6957,7 +7261,9 @@
       <c r="L123" s="1"/>
       <c r="M123" s="1"/>
       <c r="N123" s="1"/>
-      <c r="O123" s="1"/>
+      <c r="O123" s="1" t="s">
+        <v>106</v>
+      </c>
       <c r="P123" s="1"/>
       <c r="Q123" s="1"/>
       <c r="R123" s="1"/>
@@ -6965,7 +7271,7 @@
       <c r="T123" s="1"/>
       <c r="U123" s="1"/>
     </row>
-    <row r="124" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:23" x14ac:dyDescent="0.25">
       <c r="C124" s="1" t="s">
         <v>76</v>
       </c>
@@ -6975,12 +7281,12 @@
       <c r="E124" s="1"/>
       <c r="F124" s="1"/>
       <c r="G124" s="1"/>
-      <c r="H124" s="4" t="str">
+      <c r="H124" t="str">
         <f t="shared" si="0"/>
         <v>00110100</v>
       </c>
       <c r="I124" s="1"/>
-      <c r="J124" s="4" t="str" cm="1">
+      <c r="J124" t="str" cm="1">
         <f t="array" ref="J124">_xlfn.TEXTJOIN("", TRUE, MID(H124, _xlfn.SEQUENCE(LEN(H124), 1, LEN(H124), -1), 1))</f>
         <v>00101100</v>
       </c>
@@ -6988,7 +7294,9 @@
       <c r="L124" s="1"/>
       <c r="M124" s="1"/>
       <c r="N124" s="1"/>
-      <c r="O124" s="1"/>
+      <c r="O124" s="1" t="s">
+        <v>107</v>
+      </c>
       <c r="P124" s="1"/>
       <c r="Q124" s="1"/>
       <c r="R124" s="1"/>
@@ -6996,15 +7304,13 @@
       <c r="T124" s="1"/>
       <c r="U124" s="1"/>
     </row>
-    <row r="125" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:23" x14ac:dyDescent="0.25">
       <c r="C125" s="1"/>
       <c r="D125" s="1"/>
       <c r="E125" s="1"/>
       <c r="F125" s="1"/>
       <c r="G125" s="1"/>
-      <c r="H125" s="4"/>
       <c r="I125" s="1"/>
-      <c r="J125" s="4"/>
       <c r="K125" s="1"/>
       <c r="L125" s="1"/>
       <c r="M125" s="1"/>
@@ -7017,7 +7323,7 @@
       <c r="T125" s="1"/>
       <c r="U125" s="1"/>
     </row>
-    <row r="126" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>91</v>
       </c>
@@ -7037,12 +7343,12 @@
         <v>84</v>
       </c>
       <c r="G126" s="1"/>
-      <c r="H126" s="4" t="str">
+      <c r="H126" t="str">
         <f t="shared" si="0"/>
         <v>00100000</v>
       </c>
       <c r="I126" s="1"/>
-      <c r="J126" s="4" t="str" cm="1">
+      <c r="J126" t="str" cm="1">
         <f t="array" ref="J126">_xlfn.TEXTJOIN("", TRUE, MID(H126, _xlfn.SEQUENCE(LEN(H126), 1, LEN(H126), -1), 1))</f>
         <v>00000100</v>
       </c>
@@ -7050,7 +7356,9 @@
       <c r="L126" s="1"/>
       <c r="M126" s="1"/>
       <c r="N126" s="1"/>
-      <c r="O126" s="1"/>
+      <c r="O126" t="s">
+        <v>102</v>
+      </c>
       <c r="P126" s="1"/>
       <c r="Q126" s="1"/>
       <c r="R126" s="1"/>
@@ -7058,7 +7366,7 @@
       <c r="T126" s="1"/>
       <c r="U126" s="1"/>
     </row>
-    <row r="127" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:23" x14ac:dyDescent="0.25">
       <c r="C127" s="1" t="s">
         <v>21</v>
       </c>
@@ -7068,12 +7376,12 @@
       <c r="E127" s="1"/>
       <c r="F127" s="1"/>
       <c r="G127" s="1"/>
-      <c r="H127" s="4" t="str">
+      <c r="H127" t="str">
         <f t="shared" si="0"/>
         <v>00101011</v>
       </c>
       <c r="I127" s="1"/>
-      <c r="J127" s="4" t="str" cm="1">
+      <c r="J127" t="str" cm="1">
         <f t="array" ref="J127">_xlfn.TEXTJOIN("", TRUE, MID(H127, _xlfn.SEQUENCE(LEN(H127), 1, LEN(H127), -1), 1))</f>
         <v>11010100</v>
       </c>
@@ -7083,7 +7391,9 @@
       </c>
       <c r="M127" s="1"/>
       <c r="N127" s="1"/>
-      <c r="O127" s="1"/>
+      <c r="O127" s="1" t="s">
+        <v>108</v>
+      </c>
       <c r="P127" s="1"/>
       <c r="Q127" s="1"/>
       <c r="R127" s="1"/>
@@ -7091,7 +7401,7 @@
       <c r="T127" s="1"/>
       <c r="U127" s="1"/>
     </row>
-    <row r="128" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:23" x14ac:dyDescent="0.25">
       <c r="C128" s="1" t="s">
         <v>25</v>
       </c>
@@ -7101,12 +7411,12 @@
       <c r="E128" s="1"/>
       <c r="F128" s="1"/>
       <c r="G128" s="1"/>
-      <c r="H128" s="4" t="str">
+      <c r="H128" t="str">
         <f t="shared" si="0"/>
         <v>00101101</v>
       </c>
       <c r="I128" s="1"/>
-      <c r="J128" s="4" t="str" cm="1">
+      <c r="J128" t="str" cm="1">
         <f t="array" ref="J128">_xlfn.TEXTJOIN("", TRUE, MID(H128, _xlfn.SEQUENCE(LEN(H128), 1, LEN(H128), -1), 1))</f>
         <v>10110100</v>
       </c>
@@ -7114,7 +7424,9 @@
       <c r="L128" s="1"/>
       <c r="M128" s="1"/>
       <c r="N128" s="1"/>
-      <c r="O128" s="1"/>
+      <c r="O128" s="1" t="s">
+        <v>109</v>
+      </c>
       <c r="P128" s="1"/>
       <c r="Q128" s="1"/>
       <c r="R128" s="1"/>
@@ -7132,12 +7444,12 @@
       <c r="E129" s="1"/>
       <c r="F129" s="1"/>
       <c r="G129" s="1"/>
-      <c r="H129" s="4" t="str">
+      <c r="H129" t="str">
         <f t="shared" si="0"/>
         <v>01010000</v>
       </c>
       <c r="I129" s="1"/>
-      <c r="J129" s="4" t="str" cm="1">
+      <c r="J129" t="str" cm="1">
         <f t="array" ref="J129">_xlfn.TEXTJOIN("", TRUE, MID(H129, _xlfn.SEQUENCE(LEN(H129), 1, LEN(H129), -1), 1))</f>
         <v>00001010</v>
       </c>
@@ -7145,7 +7457,9 @@
       <c r="L129" s="1"/>
       <c r="M129" s="1"/>
       <c r="N129" s="1"/>
-      <c r="O129" s="1"/>
+      <c r="O129" s="1" t="s">
+        <v>110</v>
+      </c>
       <c r="P129" s="1"/>
       <c r="Q129" s="1"/>
       <c r="R129" s="1"/>
@@ -7159,9 +7473,7 @@
       <c r="E130" s="1"/>
       <c r="F130" s="1"/>
       <c r="G130" s="1"/>
-      <c r="H130" s="4"/>
       <c r="I130" s="1"/>
-      <c r="J130" s="4"/>
       <c r="K130" s="1"/>
       <c r="L130" s="1"/>
       <c r="M130" s="1"/>
@@ -7190,12 +7502,12 @@
       <c r="E131" s="1"/>
       <c r="F131" s="1"/>
       <c r="G131" s="1"/>
-      <c r="H131" s="4" t="str">
+      <c r="H131" t="str">
         <f t="shared" si="0"/>
         <v>00000000</v>
       </c>
       <c r="I131" s="1"/>
-      <c r="J131" s="4" t="str" cm="1">
+      <c r="J131" t="str" cm="1">
         <f t="array" ref="J131">_xlfn.TEXTJOIN("", TRUE, MID(H131, _xlfn.SEQUENCE(LEN(H131), 1, LEN(H131), -1), 1))</f>
         <v>00000000</v>
       </c>
@@ -7221,12 +7533,12 @@
       <c r="E132" s="1"/>
       <c r="F132" s="1"/>
       <c r="G132" s="1"/>
-      <c r="H132" s="4" t="str">
+      <c r="H132" t="str">
         <f t="shared" si="0"/>
         <v>11101000</v>
       </c>
       <c r="I132" s="1"/>
-      <c r="J132" s="4" t="str" cm="1">
+      <c r="J132" t="str" cm="1">
         <f t="array" ref="J132">_xlfn.TEXTJOIN("", TRUE, MID(H132, _xlfn.SEQUENCE(LEN(H132), 1, LEN(H132), -1), 1))</f>
         <v>00010111</v>
       </c>
@@ -7251,12 +7563,12 @@
       <c r="G133" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="H133" s="4" t="str">
+      <c r="H133" t="str">
         <f t="shared" si="0"/>
         <v>10100000</v>
       </c>
       <c r="I133" s="1"/>
-      <c r="J133" s="4" t="str" cm="1">
+      <c r="J133" t="str" cm="1">
         <f t="array" ref="J133">_xlfn.TEXTJOIN("", TRUE, MID(H133, _xlfn.SEQUENCE(LEN(H133), 1, LEN(H133), -1), 1))</f>
         <v>00000101</v>
       </c>
@@ -7269,9 +7581,7 @@
       <c r="E134" s="1"/>
       <c r="F134" s="1"/>
       <c r="G134" s="1"/>
-      <c r="H134" s="4"/>
       <c r="I134" s="1"/>
-      <c r="J134" s="4"/>
       <c r="K134" s="1"/>
       <c r="L134" s="1"/>
       <c r="M134" s="1"/>
@@ -7290,12 +7600,12 @@
       <c r="E135" s="1"/>
       <c r="F135" s="1"/>
       <c r="G135" s="1"/>
-      <c r="H135" s="4" t="str">
+      <c r="H135" t="str">
         <f t="shared" si="0"/>
         <v>00000000</v>
       </c>
       <c r="I135" s="1"/>
-      <c r="J135" s="4" t="str" cm="1">
+      <c r="J135" t="str" cm="1">
         <f t="array" ref="J135">_xlfn.TEXTJOIN("", TRUE, MID(H135, _xlfn.SEQUENCE(LEN(H135), 1, LEN(H135), -1), 1))</f>
         <v>00000000</v>
       </c>
@@ -7314,12 +7624,12 @@
       <c r="E136" s="1"/>
       <c r="F136" s="1"/>
       <c r="G136" s="1"/>
-      <c r="H136" s="4" t="str">
+      <c r="H136" t="str">
         <f t="shared" si="0"/>
         <v>00000011</v>
       </c>
       <c r="I136" s="1"/>
-      <c r="J136" s="4" t="str" cm="1">
+      <c r="J136" t="str" cm="1">
         <f t="array" ref="J136">_xlfn.TEXTJOIN("", TRUE, MID(H136, _xlfn.SEQUENCE(LEN(H136), 1, LEN(H136), -1), 1))</f>
         <v>11000000</v>
       </c>
@@ -7344,12 +7654,12 @@
       <c r="G137" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="H137" s="4" t="str">
+      <c r="H137" t="str">
         <f t="shared" si="0"/>
         <v>10000110</v>
       </c>
       <c r="I137" s="1"/>
-      <c r="J137" s="4" t="str" cm="1">
+      <c r="J137" t="str" cm="1">
         <f t="array" ref="J137">_xlfn.TEXTJOIN("", TRUE, MID(H137, _xlfn.SEQUENCE(LEN(H137), 1, LEN(H137), -1), 1))</f>
         <v>01100001</v>
       </c>
@@ -7364,9 +7674,7 @@
       <c r="E138" s="1"/>
       <c r="F138" s="1"/>
       <c r="G138" s="1"/>
-      <c r="H138" s="4"/>
       <c r="I138" s="1"/>
-      <c r="J138" s="4"/>
       <c r="K138" s="1"/>
       <c r="L138" s="1"/>
       <c r="M138" s="1"/>
@@ -7389,12 +7697,12 @@
         <v>84</v>
       </c>
       <c r="G139" s="1"/>
-      <c r="H139" s="4" t="str">
+      <c r="H139" t="str">
         <f t="shared" si="0"/>
         <v>00000000</v>
       </c>
       <c r="I139" s="1"/>
-      <c r="J139" s="4" t="str" cm="1">
+      <c r="J139" t="str" cm="1">
         <f t="array" ref="J139">_xlfn.TEXTJOIN("", TRUE, MID(H139, _xlfn.SEQUENCE(LEN(H139), 1, LEN(H139), -1), 1))</f>
         <v>00000000</v>
       </c>
@@ -7419,12 +7727,12 @@
       <c r="G140" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="H140" s="4" t="str">
+      <c r="H140" t="str">
         <f t="shared" si="0"/>
         <v>00000001</v>
       </c>
       <c r="I140" s="1"/>
-      <c r="J140" s="4" t="str" cm="1">
+      <c r="J140" t="str" cm="1">
         <f t="array" ref="J140">_xlfn.TEXTJOIN("", TRUE, MID(H140, _xlfn.SEQUENCE(LEN(H140), 1, LEN(H140), -1), 1))</f>
         <v>10000000</v>
       </c>
@@ -7516,6 +7824,9 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="I34:M34"/>
+  </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>